<commit_message>
add reg, cfs, sponsors
</commit_message>
<xml_diff>
--- a/assets/misc/2025/2025_Attendance.xlsx
+++ b/assets/misc/2025/2025_Attendance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F406BC21-4AFD-4F25-B8BD-0F42F81F997C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913985B1-9953-4F5E-A991-0FC67300006C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22095" yWindow="0" windowWidth="17475" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4275" yWindow="165" windowWidth="19965" windowHeight="14895" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -749,6 +749,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="H9" s="9">
+        <f>SUM(D8:D30)</f>
+        <v>3302</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5">

</xml_diff>

<commit_message>
add reg, cfs, sponsors (#1331)
Co-authored-by: way0utwest <admin@sqlsaturday.com>
</commit_message>
<xml_diff>
--- a/assets/misc/2025/2025_Attendance.xlsx
+++ b/assets/misc/2025/2025_Attendance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F406BC21-4AFD-4F25-B8BD-0F42F81F997C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913985B1-9953-4F5E-A991-0FC67300006C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22095" yWindow="0" windowWidth="17475" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4275" yWindow="165" windowWidth="19965" windowHeight="14895" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -749,6 +749,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="H9" s="9">
+        <f>SUM(D8:D30)</f>
+        <v>3302</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5">

</xml_diff>